<commit_message>
feat(logistics): adjust manifest sealing/receive rules and tracking display
- manifest-service: allow seal without shipments; allow receive when CREATED\n- tracking-service: update VI labels, manifest.sealed status mapping, timeline notes\n- web/mobile: related UI/copy updates\n- docs: update ThaoTac.xlsx
</commit_message>
<xml_diff>
--- a/docs/Documents/ThaoTac.xlsx
+++ b/docs/Documents/ThaoTac.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bro\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\Semester 2_Year 4\New Technology\logistics-management-system\docs\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8D75307-6458-47AD-A3D6-505DA6533E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053A8CDB-3C6A-4E9B-A2AD-7E09D9786BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{0A048C3C-1687-4BA6-8BD8-435170433F60}"/>
   </bookViews>
@@ -25,17 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="36">
   <si>
     <t xml:space="preserve">Thao tác </t>
   </si>
   <si>
-    <t>Trạng thái hiển thị trên OPS</t>
-  </si>
-  <si>
-    <t>Trạng thái hiển thị trên Merchant</t>
-  </si>
-  <si>
     <t>Ghi chú chi tiết</t>
   </si>
   <si>
@@ -100,15 +94,62 @@
   </si>
   <si>
     <t>Ký nhận</t>
+  </si>
+  <si>
+    <t>Gỡ bao</t>
+  </si>
+  <si>
+    <t>Courier/Ops</t>
+  </si>
+  <si>
+    <t>Ghi nhận Vấn đề</t>
+  </si>
+  <si>
+    <t>Ghi nhận vấn đề</t>
+  </si>
+  <si>
+    <t>Vấn đề -Tên nhân viên - mã nhân viên - mã hub thao tác</t>
+  </si>
+  <si>
+    <t>Quét tồn kho</t>
+  </si>
+  <si>
+    <t>Trạng thái vận đơn hiển thị trên OPS</t>
+  </si>
+  <si>
+    <t>Trạng thái vận đơn hiển thị trên Merchant</t>
+  </si>
+  <si>
+    <t>Trạng thái tem xe</t>
+  </si>
+  <si>
+    <t>Tạo tem xe</t>
+  </si>
+  <si>
+    <t>Khởi tạo</t>
+  </si>
+  <si>
+    <t>Chờ xuất phát</t>
+  </si>
+  <si>
+    <t>Đã đến</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -135,8 +176,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,200 +493,269 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{53591E7D-5C5A-43E3-80DA-07CA030A5B69}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.08984375" customWidth="1"/>
+    <col min="4" max="4" width="34.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="48.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="D5" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
       </c>
       <c r="E5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" t="s">
-        <v>20</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="B14" t="s">
         <v>22</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D14" t="s">
         <v>22</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E14" t="s">
         <v>22</v>
       </c>
-      <c r="E10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="F14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>24</v>
       </c>
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-      <c r="E12" t="s">
-        <v>15</v>
+      <c r="B15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>